<commit_message>
actualiza acumulados 18/06/2026 17:08
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO-BILBAO-(IED)-901_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO-BILBAO-(IED)-901_CALIFICADO.xlsx
@@ -11707,7 +11707,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>LENGUAJE</t>
+          <t>MATEMÁTICAS</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -11725,9 +11725,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -11735,9 +11735,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
@@ -11755,9 +11755,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="R45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="R45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="S45" s="2" t="inlineStr">
@@ -11765,9 +11765,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="T45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -11775,9 +11775,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W45" s="2" t="inlineStr">
@@ -11805,9 +11805,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="AB45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AB45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AC45" s="2" t="inlineStr">
@@ -11845,9 +11845,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="AJ45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AJ45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AK45" s="2" t="inlineStr">
@@ -11855,9 +11855,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="AL45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AL45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AM45" s="2" t="inlineStr">
@@ -11885,9 +11885,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="AR45" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="AR45" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AS45" s="2" t="inlineStr">
@@ -11895,9 +11895,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="AT45" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="AT45" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AU45" s="2" t="inlineStr">
@@ -11905,9 +11905,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="AV45" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AV45" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AW45" s="5">
@@ -18016,7 +18016,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>LENGUAJE</t>
+          <t>MATEMÁTICAS</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -18034,9 +18034,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr">
@@ -18044,9 +18044,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="N70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
@@ -18064,9 +18064,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="R70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="S70" s="2" t="inlineStr">
@@ -18074,9 +18074,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="T70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="T70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="U70" s="2" t="inlineStr">
@@ -18084,9 +18084,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="V70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="V70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="W70" s="2" t="inlineStr">
@@ -18114,9 +18114,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="AB70" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="AB70" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AC70" s="2" t="inlineStr">
@@ -18134,9 +18134,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="AF70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AF70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AG70" s="2" t="inlineStr">
@@ -18164,9 +18164,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="AL70" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="AL70" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="AM70" s="2" t="inlineStr">
@@ -18194,9 +18194,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="AR70" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="AR70" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="AS70" s="2" t="inlineStr"/>

</xml_diff>